<commit_message>
Deploying to main from @ open-resource-discovery/specification@37155aaf6524c2ef80a95b85c30b4a56fd8bb350 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-181/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-181/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="209">
   <si>
     <t>Entity Name</t>
   </si>
@@ -433,6 +433,9 @@
     <t>systemTypes</t>
   </si>
   <si>
+    <t>array&lt;SystemTypeIntegrationAspect&gt;</t>
+  </si>
+  <si>
     <t>apiResources</t>
   </si>
   <si>
@@ -487,6 +490,12 @@
     <t>Capability Integration Aspect</t>
   </si>
   <si>
+    <t>System Type Integration Aspect</t>
+  </si>
+  <si>
+    <t>systemNamespace</t>
+  </si>
+  <si>
     <t>Vendor</t>
   </si>
   <si>
@@ -521,9 +530,6 @@
   </si>
   <si>
     <t>System Type</t>
-  </si>
-  <si>
-    <t>systemNamespace</t>
   </si>
   <si>
     <t>System Version</t>
@@ -1008,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D478"/>
+  <dimension ref="A1:D480"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5894,7 +5900,7 @@
         <v>0</v>
       </c>
       <c r="D349" t="s">
-        <v>9</v>
+        <v>140</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
@@ -5902,13 +5908,13 @@
         <v>137</v>
       </c>
       <c r="B350" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C350" t="b">
         <v>0</v>
       </c>
       <c r="D350" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
@@ -5916,13 +5922,13 @@
         <v>137</v>
       </c>
       <c r="B351" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C351" t="b">
         <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
@@ -5930,13 +5936,13 @@
         <v>137</v>
       </c>
       <c r="B352" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C352" t="b">
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
@@ -5955,7 +5961,7 @@
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B354" t="s">
         <v>5</v>
@@ -5969,10 +5975,10 @@
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B355" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C355" t="b">
         <v>0</v>
@@ -5983,21 +5989,21 @@
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B356" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C356" t="b">
         <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B357" t="s">
         <v>32</v>
@@ -6011,7 +6017,7 @@
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B358" t="s">
         <v>5</v>
@@ -6025,10 +6031,10 @@
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B359" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C359" t="b">
         <v>0</v>
@@ -6039,24 +6045,24 @@
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B360" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C360" t="b">
         <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B361" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C361" t="b">
         <v>0</v>
@@ -6067,7 +6073,7 @@
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B362" t="s">
         <v>32</v>
@@ -6081,10 +6087,10 @@
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B363" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C363" t="b">
         <v>1</v>
@@ -6095,10 +6101,10 @@
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B364" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C364" t="b">
         <v>1</v>
@@ -6109,7 +6115,7 @@
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B365" t="s">
         <v>5</v>
@@ -6123,10 +6129,10 @@
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B366" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C366" t="b">
         <v>0</v>
@@ -6137,7 +6143,7 @@
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B367" t="s">
         <v>32</v>
@@ -6151,10 +6157,10 @@
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B368" t="s">
-        <v>5</v>
+        <v>160</v>
       </c>
       <c r="C368" t="b">
         <v>1</v>
@@ -6165,13 +6171,13 @@
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B369" t="s">
-        <v>10</v>
+        <v>148</v>
       </c>
       <c r="C369" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D369" t="s">
         <v>6</v>
@@ -6179,94 +6185,94 @@
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B370" t="s">
-        <v>159</v>
+        <v>5</v>
       </c>
       <c r="C370" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D370" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B371" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C371" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D371" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B372" t="s">
-        <v>32</v>
+        <v>162</v>
       </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B373" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C373" t="b">
         <v>0</v>
       </c>
       <c r="D373" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B374" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C374" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D374" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B375" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="C375" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D375" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B376" t="s">
-        <v>161</v>
+        <v>13</v>
       </c>
       <c r="C376" t="b">
         <v>1</v>
@@ -6277,13 +6283,13 @@
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B377" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="C377" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D377" t="s">
         <v>6</v>
@@ -6291,13 +6297,13 @@
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B378" t="s">
-        <v>99</v>
+        <v>164</v>
       </c>
       <c r="C378" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D378" t="s">
         <v>6</v>
@@ -6305,13 +6311,13 @@
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B379" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C379" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D379" t="s">
         <v>6</v>
@@ -6319,13 +6325,13 @@
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B380" t="s">
         <v>99</v>
       </c>
       <c r="C380" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D380" t="s">
         <v>6</v>
@@ -6333,13 +6339,13 @@
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B381" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C381" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D381" t="s">
         <v>6</v>
@@ -6347,10 +6353,10 @@
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B382" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="C382" t="b">
         <v>1</v>
@@ -6361,13 +6367,13 @@
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B383" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C383" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D383" t="s">
         <v>6</v>
@@ -6375,13 +6381,13 @@
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B384" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C384" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D384" t="s">
         <v>6</v>
@@ -6389,10 +6395,10 @@
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B385" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C385" t="b">
         <v>1</v>
@@ -6403,13 +6409,13 @@
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B386" t="s">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="C386" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D386" t="s">
         <v>6</v>
@@ -6417,13 +6423,13 @@
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B387" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="C387" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D387" t="s">
         <v>6</v>
@@ -6431,10 +6437,10 @@
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B388" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C388" t="b">
         <v>1</v>
@@ -6445,13 +6451,13 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B389" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C389" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D389" t="s">
         <v>6</v>
@@ -6459,13 +6465,13 @@
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B390" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C390" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D390" t="s">
         <v>6</v>
@@ -6473,10 +6479,10 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B391" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C391" t="b">
         <v>1</v>
@@ -6487,13 +6493,13 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B392" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C392" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D392" t="s">
         <v>6</v>
@@ -6501,13 +6507,13 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B393" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C393" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D393" t="s">
         <v>6</v>
@@ -6515,10 +6521,10 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B394" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C394" t="b">
         <v>1</v>
@@ -6529,10 +6535,10 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B395" t="s">
-        <v>168</v>
+        <v>115</v>
       </c>
       <c r="C395" t="b">
         <v>0</v>
@@ -6543,13 +6549,13 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B396" t="s">
-        <v>7</v>
+        <v>99</v>
       </c>
       <c r="C396" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D396" t="s">
         <v>6</v>
@@ -6557,80 +6563,80 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B397" t="s">
-        <v>8</v>
+        <v>171</v>
       </c>
       <c r="C397" t="b">
         <v>0</v>
       </c>
       <c r="D397" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B398" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C398" t="b">
         <v>0</v>
       </c>
       <c r="D398" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B399" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="C399" t="b">
         <v>0</v>
       </c>
       <c r="D399" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B400" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C400" t="b">
         <v>0</v>
       </c>
       <c r="D400" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B401" t="s">
-        <v>170</v>
+        <v>34</v>
       </c>
       <c r="C401" t="b">
         <v>0</v>
       </c>
       <c r="D401" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B402" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C402" t="b">
         <v>0</v>
@@ -6641,167 +6647,167 @@
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B403" t="s">
-        <v>32</v>
+        <v>160</v>
       </c>
       <c r="C403" t="b">
         <v>0</v>
       </c>
       <c r="D403" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B404" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="C404" t="b">
         <v>0</v>
       </c>
       <c r="D404" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B405" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C405" t="b">
         <v>0</v>
       </c>
       <c r="D405" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B406" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="C406" t="b">
         <v>0</v>
       </c>
       <c r="D406" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B407" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C407" t="b">
         <v>0</v>
       </c>
       <c r="D407" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B408" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C408" t="b">
         <v>0</v>
       </c>
       <c r="D408" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B409" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
       </c>
       <c r="D409" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B410" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="C410" t="b">
         <v>0</v>
       </c>
       <c r="D410" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B411" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C411" t="b">
         <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B412" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="C412" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B413" t="s">
-        <v>115</v>
+        <v>31</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
       </c>
       <c r="D413" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B414" t="s">
-        <v>173</v>
+        <v>97</v>
       </c>
       <c r="C414" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D414" t="s">
         <v>6</v>
@@ -6812,10 +6818,10 @@
         <v>174</v>
       </c>
       <c r="B415" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C415" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D415" t="s">
         <v>6</v>
@@ -6826,7 +6832,7 @@
         <v>174</v>
       </c>
       <c r="B416" t="s">
-        <v>115</v>
+        <v>175</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
@@ -6837,13 +6843,13 @@
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B417" t="s">
-        <v>173</v>
+        <v>97</v>
       </c>
       <c r="C417" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D417" t="s">
         <v>6</v>
@@ -6851,10 +6857,10 @@
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B418" t="s">
-        <v>175</v>
+        <v>115</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
@@ -6868,10 +6874,10 @@
         <v>176</v>
       </c>
       <c r="B419" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C419" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D419" t="s">
         <v>6</v>
@@ -6882,10 +6888,10 @@
         <v>176</v>
       </c>
       <c r="B420" t="s">
-        <v>10</v>
+        <v>177</v>
       </c>
       <c r="C420" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D420" t="s">
         <v>6</v>
@@ -6893,13 +6899,13 @@
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B421" t="s">
-        <v>12</v>
+        <v>179</v>
       </c>
       <c r="C421" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D421" t="s">
         <v>6</v>
@@ -6907,83 +6913,83 @@
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B422" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C422" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D422" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B423" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B424" t="s">
-        <v>178</v>
+        <v>32</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
       </c>
       <c r="D424" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B425" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="C425" t="b">
         <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B426" t="s">
         <v>180</v>
       </c>
       <c r="C426" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D426" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B427" t="s">
-        <v>177</v>
+        <v>38</v>
       </c>
       <c r="C427" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D427" t="s">
         <v>6</v>
@@ -6991,10 +6997,10 @@
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B428" t="s">
-        <v>10</v>
+        <v>182</v>
       </c>
       <c r="C428" t="b">
         <v>1</v>
@@ -7005,13 +7011,13 @@
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
+        <v>181</v>
+      </c>
+      <c r="B429" t="s">
         <v>179</v>
       </c>
-      <c r="B429" t="s">
-        <v>12</v>
-      </c>
       <c r="C429" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D429" t="s">
         <v>6</v>
@@ -7019,80 +7025,80 @@
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B430" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C430" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D430" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B431" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C431" t="b">
         <v>0</v>
       </c>
       <c r="D431" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B432" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C432" t="b">
         <v>0</v>
       </c>
       <c r="D432" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B433" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="C433" t="b">
         <v>0</v>
       </c>
       <c r="D433" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B434" t="s">
-        <v>181</v>
+        <v>46</v>
       </c>
       <c r="C434" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D434" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B435" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="C435" t="b">
         <v>0</v>
@@ -7103,58 +7109,58 @@
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>182</v>
+        <v>84</v>
       </c>
       <c r="B436" t="s">
         <v>183</v>
       </c>
       <c r="C436" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D436" t="s">
-        <v>184</v>
+        <v>6</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>182</v>
+        <v>84</v>
       </c>
       <c r="B437" t="s">
-        <v>185</v>
+        <v>12</v>
       </c>
       <c r="C437" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D437" t="s">
-        <v>186</v>
+        <v>6</v>
       </c>
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B438" t="s">
-        <v>5</v>
+        <v>185</v>
       </c>
       <c r="C438" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D438" t="s">
-        <v>6</v>
+        <v>186</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
+        <v>184</v>
+      </c>
+      <c r="B439" t="s">
         <v>187</v>
       </c>
-      <c r="B439" t="s">
+      <c r="C439" t="b">
+        <v>1</v>
+      </c>
+      <c r="D439" t="s">
         <v>188</v>
-      </c>
-      <c r="C439" t="b">
-        <v>1</v>
-      </c>
-      <c r="D439" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
@@ -7176,7 +7182,7 @@
         <v>189</v>
       </c>
       <c r="B441" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C441" t="b">
         <v>1</v>
@@ -7187,10 +7193,10 @@
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B442" t="s">
-        <v>97</v>
+        <v>5</v>
       </c>
       <c r="C442" t="b">
         <v>1</v>
@@ -7201,10 +7207,10 @@
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
+        <v>191</v>
+      </c>
+      <c r="B443" t="s">
         <v>190</v>
-      </c>
-      <c r="B443" t="s">
-        <v>191</v>
       </c>
       <c r="C443" t="b">
         <v>1</v>
@@ -7246,7 +7252,7 @@
         <v>194</v>
       </c>
       <c r="B446" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C446" t="b">
         <v>1</v>
@@ -7257,10 +7263,10 @@
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
+        <v>194</v>
+      </c>
+      <c r="B447" t="s">
         <v>195</v>
-      </c>
-      <c r="B447" t="s">
-        <v>5</v>
       </c>
       <c r="C447" t="b">
         <v>1</v>
@@ -7274,7 +7280,7 @@
         <v>196</v>
       </c>
       <c r="B448" t="s">
-        <v>197</v>
+        <v>5</v>
       </c>
       <c r="C448" t="b">
         <v>1</v>
@@ -7285,7 +7291,7 @@
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B449" t="s">
         <v>5</v>
@@ -7305,7 +7311,7 @@
         <v>199</v>
       </c>
       <c r="C450" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D450" t="s">
         <v>6</v>
@@ -7330,7 +7336,7 @@
         <v>200</v>
       </c>
       <c r="B452" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C452" t="b">
         <v>0</v>
@@ -7341,7 +7347,7 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B453" t="s">
         <v>5</v>
@@ -7355,10 +7361,10 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
+        <v>202</v>
+      </c>
+      <c r="B454" t="s">
         <v>201</v>
-      </c>
-      <c r="B454" t="s">
-        <v>199</v>
       </c>
       <c r="C454" t="b">
         <v>0</v>
@@ -7369,7 +7375,7 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B455" t="s">
         <v>5</v>
@@ -7383,10 +7389,10 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B456" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C456" t="b">
         <v>0</v>
@@ -7397,7 +7403,7 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B457" t="s">
         <v>5</v>
@@ -7414,7 +7420,7 @@
         <v>204</v>
       </c>
       <c r="B458" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C458" t="b">
         <v>0</v>
@@ -7425,13 +7431,13 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B459" t="s">
-        <v>180</v>
+        <v>5</v>
       </c>
       <c r="C459" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D459" t="s">
         <v>6</v>
@@ -7439,10 +7445,10 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B460" t="s">
-        <v>177</v>
+        <v>5</v>
       </c>
       <c r="C460" t="b">
         <v>0</v>
@@ -7453,13 +7459,13 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B461" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="C461" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D461" t="s">
         <v>6</v>
@@ -7467,10 +7473,10 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B462" t="s">
-        <v>12</v>
+        <v>179</v>
       </c>
       <c r="C462" t="b">
         <v>0</v>
@@ -7484,7 +7490,7 @@
         <v>206</v>
       </c>
       <c r="B463" t="s">
-        <v>5</v>
+        <v>207</v>
       </c>
       <c r="C463" t="b">
         <v>1</v>
@@ -7498,7 +7504,7 @@
         <v>206</v>
       </c>
       <c r="B464" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C464" t="b">
         <v>0</v>
@@ -7509,27 +7515,27 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B465" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C465" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D465" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B466" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C466" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D466" t="s">
         <v>6</v>
@@ -7537,24 +7543,24 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B467" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C467" t="b">
         <v>0</v>
       </c>
       <c r="D467" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B468" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C468" t="b">
         <v>1</v>
@@ -7565,13 +7571,13 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B469" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="C469" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7579,24 +7585,24 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B470" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="C470" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D470" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B471" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="C471" t="b">
         <v>1</v>
@@ -7607,24 +7613,24 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B472" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C472" t="b">
         <v>0</v>
       </c>
       <c r="D472" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B473" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="C473" t="b">
         <v>1</v>
@@ -7635,13 +7641,13 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B474" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="C474" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D474" t="s">
         <v>6</v>
@@ -7649,57 +7655,85 @@
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B475" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="C475" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D475" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B476" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="C476" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D476" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B477" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C477" t="b">
         <v>0</v>
       </c>
       <c r="D477" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B478" t="s">
+        <v>31</v>
+      </c>
+      <c r="C478" t="b">
+        <v>0</v>
+      </c>
+      <c r="D478" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="479" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A479" t="s">
+        <v>208</v>
+      </c>
+      <c r="B479" t="s">
+        <v>32</v>
+      </c>
+      <c r="C479" t="b">
+        <v>0</v>
+      </c>
+      <c r="D479" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="480" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A480" t="s">
+        <v>208</v>
+      </c>
+      <c r="B480" t="s">
         <v>34</v>
       </c>
-      <c r="C478" t="b">
-        <v>0</v>
-      </c>
-      <c r="D478" t="s">
+      <c r="C480" t="b">
+        <v>0</v>
+      </c>
+      <c r="D480" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploying to main from @ open-resource-discovery/specification@bc350af42baf2167238a53f3589dff29eda5985e 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-181/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-181/spec-v1/interfaces/Document.xlsx
@@ -430,28 +430,28 @@
     <t>supportMultipleProviders</t>
   </si>
   <si>
+    <t>apiResources</t>
+  </si>
+  <si>
+    <t>array&lt;ApiResourceIntegrationAspect&gt;</t>
+  </si>
+  <si>
+    <t>eventResources</t>
+  </si>
+  <si>
+    <t>array&lt;EventResourceIntegrationAspect&gt;</t>
+  </si>
+  <si>
+    <t>capabilities</t>
+  </si>
+  <si>
+    <t>array&lt;CapabilityIntegrationAspect&gt;</t>
+  </si>
+  <si>
     <t>systemTypes</t>
   </si>
   <si>
     <t>array&lt;SystemTypeIntegrationAspect&gt;</t>
-  </si>
-  <si>
-    <t>apiResources</t>
-  </si>
-  <si>
-    <t>array&lt;ApiResourceIntegrationAspect&gt;</t>
-  </si>
-  <si>
-    <t>eventResources</t>
-  </si>
-  <si>
-    <t>array&lt;EventResourceIntegrationAspect&gt;</t>
-  </si>
-  <si>
-    <t>capabilities</t>
-  </si>
-  <si>
-    <t>array&lt;CapabilityIntegrationAspect&gt;</t>
   </si>
   <si>
     <t>Api Resource Integration Aspect</t>
@@ -6174,7 +6174,7 @@
         <v>159</v>
       </c>
       <c r="B369" t="s">
-        <v>148</v>
+        <v>54</v>
       </c>
       <c r="C369" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Deploying to main from @ open-resource-discovery/specification@05d626c7961faf6005959a5d492d9ffb3a0c7722 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-181/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-181/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1483" uniqueCount="212">
   <si>
     <t>Entity Name</t>
   </si>
@@ -490,10 +490,19 @@
     <t>Capability Integration Aspect</t>
   </si>
   <si>
+    <t>array&lt;CapabilityIntegrationAspectSubset&gt;</t>
+  </si>
+  <si>
     <t>System Type Integration Aspect</t>
   </si>
   <si>
     <t>systemNamespace</t>
+  </si>
+  <si>
+    <t>Capability Integration Aspect Subset</t>
+  </si>
+  <si>
+    <t>skillName</t>
   </si>
   <si>
     <t>Vendor</t>
@@ -1014,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D480"/>
+  <dimension ref="A1:D494"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5222,13 +5231,13 @@
         <v>127</v>
       </c>
       <c r="B301" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C301" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D301" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
@@ -5236,10 +5245,10 @@
         <v>127</v>
       </c>
       <c r="B302" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C302" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D302" t="s">
         <v>6</v>
@@ -5250,10 +5259,10 @@
         <v>127</v>
       </c>
       <c r="B303" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C303" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D303" t="s">
         <v>6</v>
@@ -5264,7 +5273,7 @@
         <v>127</v>
       </c>
       <c r="B304" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C304" t="b">
         <v>1</v>
@@ -5278,13 +5287,13 @@
         <v>127</v>
       </c>
       <c r="B305" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C305" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D305" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
@@ -5292,13 +5301,13 @@
         <v>127</v>
       </c>
       <c r="B306" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C306" t="b">
         <v>0</v>
       </c>
       <c r="D306" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
@@ -5306,13 +5315,13 @@
         <v>127</v>
       </c>
       <c r="B307" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="C307" t="b">
         <v>0</v>
       </c>
       <c r="D307" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
@@ -5320,13 +5329,13 @@
         <v>127</v>
       </c>
       <c r="B308" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="C308" t="b">
         <v>0</v>
       </c>
       <c r="D308" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
@@ -5334,13 +5343,13 @@
         <v>127</v>
       </c>
       <c r="B309" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C309" t="b">
         <v>0</v>
       </c>
       <c r="D309" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
@@ -5348,13 +5357,13 @@
         <v>127</v>
       </c>
       <c r="B310" t="s">
-        <v>128</v>
+        <v>60</v>
       </c>
       <c r="C310" t="b">
         <v>0</v>
       </c>
       <c r="D310" t="s">
-        <v>129</v>
+        <v>6</v>
       </c>
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
@@ -5362,13 +5371,13 @@
         <v>127</v>
       </c>
       <c r="B311" t="s">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="C311" t="b">
         <v>0</v>
       </c>
       <c r="D311" t="s">
-        <v>130</v>
+        <v>9</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.25">
@@ -5376,13 +5385,13 @@
         <v>127</v>
       </c>
       <c r="B312" t="s">
-        <v>19</v>
+        <v>62</v>
       </c>
       <c r="C312" t="b">
         <v>0</v>
       </c>
       <c r="D312" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
@@ -5390,7 +5399,7 @@
         <v>127</v>
       </c>
       <c r="B313" t="s">
-        <v>31</v>
+        <v>92</v>
       </c>
       <c r="C313" t="b">
         <v>0</v>
@@ -5404,13 +5413,13 @@
         <v>127</v>
       </c>
       <c r="B314" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="C314" t="b">
         <v>0</v>
       </c>
       <c r="D314" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
@@ -5418,13 +5427,13 @@
         <v>127</v>
       </c>
       <c r="B315" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="C315" t="b">
         <v>0</v>
       </c>
       <c r="D315" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
@@ -5432,192 +5441,192 @@
         <v>127</v>
       </c>
       <c r="B316" t="s">
-        <v>85</v>
+        <v>128</v>
       </c>
       <c r="C316" t="b">
         <v>0</v>
       </c>
       <c r="D316" t="s">
-        <v>51</v>
+        <v>129</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B317" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="C317" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B318" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="C318" t="b">
         <v>0</v>
       </c>
       <c r="D318" t="s">
-        <v>6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B319" t="s">
-        <v>98</v>
+        <v>19</v>
       </c>
       <c r="C319" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D319" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B320" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="C320" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D320" t="s">
-        <v>6</v>
+        <v>84</v>
       </c>
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B321" t="s">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="C321" t="b">
         <v>0</v>
       </c>
       <c r="D321" t="s">
-        <v>101</v>
+        <v>9</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B322" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C322" t="b">
         <v>0</v>
       </c>
       <c r="D322" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B323" t="s">
-        <v>116</v>
+        <v>29</v>
       </c>
       <c r="C323" t="b">
         <v>0</v>
       </c>
       <c r="D323" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B324" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C324" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D324" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B325" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C325" t="b">
         <v>0</v>
       </c>
       <c r="D325" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B326" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
       </c>
       <c r="D326" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B327" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C327" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D327" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B328" t="s">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="C328" t="b">
         <v>0</v>
       </c>
       <c r="D328" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B329" t="s">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="C329" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D329" t="s">
         <v>6</v>
@@ -5625,13 +5634,13 @@
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B330" t="s">
-        <v>45</v>
+        <v>115</v>
       </c>
       <c r="C330" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D330" t="s">
         <v>6</v>
@@ -5639,24 +5648,24 @@
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B331" t="s">
-        <v>46</v>
+        <v>98</v>
       </c>
       <c r="C331" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D331" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B332" t="s">
-        <v>13</v>
+        <v>99</v>
       </c>
       <c r="C332" t="b">
         <v>1</v>
@@ -5667,27 +5676,27 @@
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B333" t="s">
-        <v>37</v>
+        <v>100</v>
       </c>
       <c r="C333" t="b">
         <v>0</v>
       </c>
       <c r="D333" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B334" t="s">
         <v>38</v>
       </c>
       <c r="C334" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D334" t="s">
         <v>6</v>
@@ -5695,13 +5704,13 @@
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B335" t="s">
-        <v>52</v>
+        <v>116</v>
       </c>
       <c r="C335" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D335" t="s">
         <v>6</v>
@@ -5712,10 +5721,10 @@
         <v>132</v>
       </c>
       <c r="B336" t="s">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="C336" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D336" t="s">
         <v>6</v>
@@ -5726,13 +5735,13 @@
         <v>132</v>
       </c>
       <c r="B337" t="s">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="C337" t="b">
         <v>0</v>
       </c>
       <c r="D337" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
@@ -5740,13 +5749,13 @@
         <v>132</v>
       </c>
       <c r="B338" t="s">
-        <v>133</v>
+        <v>8</v>
       </c>
       <c r="C338" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D338" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
@@ -5754,13 +5763,13 @@
         <v>132</v>
       </c>
       <c r="B339" t="s">
-        <v>134</v>
+        <v>10</v>
       </c>
       <c r="C339" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D339" t="s">
-        <v>135</v>
+        <v>6</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
@@ -5768,13 +5777,13 @@
         <v>132</v>
       </c>
       <c r="B340" t="s">
-        <v>136</v>
+        <v>11</v>
       </c>
       <c r="C340" t="b">
         <v>0</v>
       </c>
       <c r="D340" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
@@ -5782,13 +5791,13 @@
         <v>132</v>
       </c>
       <c r="B341" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C341" t="b">
         <v>0</v>
       </c>
       <c r="D341" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
@@ -5796,13 +5805,13 @@
         <v>132</v>
       </c>
       <c r="B342" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="C342" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D342" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
@@ -5810,13 +5819,13 @@
         <v>132</v>
       </c>
       <c r="B343" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="C343" t="b">
         <v>0</v>
       </c>
       <c r="D343" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
@@ -5824,21 +5833,21 @@
         <v>132</v>
       </c>
       <c r="B344" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C344" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D344" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B345" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="C345" t="b">
         <v>0</v>
@@ -5849,13 +5858,13 @@
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B346" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="C346" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D346" t="s">
         <v>6</v>
@@ -5863,167 +5872,167 @@
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B347" t="s">
-        <v>133</v>
+        <v>52</v>
       </c>
       <c r="C347" t="b">
         <v>1</v>
       </c>
       <c r="D347" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B348" t="s">
-        <v>138</v>
+        <v>60</v>
       </c>
       <c r="C348" t="b">
         <v>0</v>
       </c>
       <c r="D348" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B349" t="s">
-        <v>139</v>
+        <v>61</v>
       </c>
       <c r="C349" t="b">
         <v>0</v>
       </c>
       <c r="D349" t="s">
-        <v>140</v>
+        <v>9</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B350" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="C350" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D350" t="s">
-        <v>142</v>
+        <v>51</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B351" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="C351" t="b">
         <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B352" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C352" t="b">
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>146</v>
+        <v>9</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B353" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C353" t="b">
         <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="B354" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C354" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D354" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="B355" t="s">
-        <v>148</v>
+        <v>32</v>
       </c>
       <c r="C355" t="b">
         <v>0</v>
       </c>
       <c r="D355" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="B356" t="s">
-        <v>149</v>
+        <v>34</v>
       </c>
       <c r="C356" t="b">
         <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>150</v>
+        <v>35</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="B357" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C357" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D357" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="B358" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C358" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D358" t="s">
         <v>6</v>
@@ -6031,111 +6040,111 @@
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="B359" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="C359" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D359" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="B360" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="C360" t="b">
         <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>152</v>
+        <v>51</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="B361" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="C361" t="b">
         <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>9</v>
+        <v>140</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="B362" t="s">
-        <v>32</v>
+        <v>141</v>
       </c>
       <c r="C362" t="b">
         <v>0</v>
       </c>
       <c r="D362" t="s">
-        <v>33</v>
+        <v>142</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="B363" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="C363" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D363" t="s">
-        <v>6</v>
+        <v>144</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
       <c r="B364" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="C364" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D364" t="s">
-        <v>6</v>
+        <v>146</v>
       </c>
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="B365" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C365" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D365" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B366" t="s">
-        <v>148</v>
+        <v>5</v>
       </c>
       <c r="C366" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D366" t="s">
         <v>6</v>
@@ -6143,49 +6152,49 @@
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B367" t="s">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="C367" t="b">
         <v>0</v>
       </c>
       <c r="D367" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="B368" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="C368" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D368" t="s">
-        <v>6</v>
+        <v>150</v>
       </c>
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="B369" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="C369" t="b">
         <v>0</v>
       </c>
       <c r="D369" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B370" t="s">
         <v>5</v>
@@ -6199,13 +6208,13 @@
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B371" t="s">
-        <v>10</v>
+        <v>148</v>
       </c>
       <c r="C371" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D371" t="s">
         <v>6</v>
@@ -6213,24 +6222,24 @@
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B372" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>9</v>
+        <v>152</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B373" t="s">
-        <v>31</v>
+        <v>153</v>
       </c>
       <c r="C373" t="b">
         <v>0</v>
@@ -6241,7 +6250,7 @@
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B374" t="s">
         <v>32</v>
@@ -6255,24 +6264,24 @@
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="B375" t="s">
-        <v>34</v>
+        <v>155</v>
       </c>
       <c r="C375" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D375" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="B376" t="s">
-        <v>13</v>
+        <v>157</v>
       </c>
       <c r="C376" t="b">
         <v>1</v>
@@ -6283,10 +6292,10 @@
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B377" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="C377" t="b">
         <v>1</v>
@@ -6297,13 +6306,13 @@
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B378" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="C378" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D378" t="s">
         <v>6</v>
@@ -6311,38 +6320,38 @@
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B379" t="s">
-        <v>12</v>
+        <v>149</v>
       </c>
       <c r="C379" t="b">
         <v>0</v>
       </c>
       <c r="D379" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B380" t="s">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="C380" t="b">
         <v>0</v>
       </c>
       <c r="D380" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B381" t="s">
-        <v>10</v>
+        <v>161</v>
       </c>
       <c r="C381" t="b">
         <v>1</v>
@@ -6353,13 +6362,13 @@
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B382" t="s">
-        <v>99</v>
+        <v>54</v>
       </c>
       <c r="C382" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D382" t="s">
         <v>6</v>
@@ -6367,13 +6376,13 @@
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B383" t="s">
-        <v>12</v>
+        <v>163</v>
       </c>
       <c r="C383" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D383" t="s">
         <v>6</v>
@@ -6381,10 +6390,10 @@
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B384" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C384" t="b">
         <v>1</v>
@@ -6395,10 +6404,10 @@
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B385" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C385" t="b">
         <v>1</v>
@@ -6409,66 +6418,66 @@
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B386" t="s">
-        <v>12</v>
+        <v>165</v>
       </c>
       <c r="C386" t="b">
         <v>0</v>
       </c>
       <c r="D386" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B387" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="C387" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D387" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B388" t="s">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="C388" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D388" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B389" t="s">
-        <v>115</v>
+        <v>34</v>
       </c>
       <c r="C389" t="b">
         <v>0</v>
       </c>
       <c r="D389" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B390" t="s">
-        <v>99</v>
+        <v>13</v>
       </c>
       <c r="C390" t="b">
         <v>1</v>
@@ -6479,10 +6488,10 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B391" t="s">
-        <v>97</v>
+        <v>52</v>
       </c>
       <c r="C391" t="b">
         <v>1</v>
@@ -6493,13 +6502,13 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B392" t="s">
-        <v>115</v>
+        <v>167</v>
       </c>
       <c r="C392" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D392" t="s">
         <v>6</v>
@@ -6507,13 +6516,13 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B393" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C393" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D393" t="s">
         <v>6</v>
@@ -6521,13 +6530,13 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B394" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C394" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D394" t="s">
         <v>6</v>
@@ -6535,13 +6544,13 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B395" t="s">
-        <v>115</v>
+        <v>10</v>
       </c>
       <c r="C395" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D395" t="s">
         <v>6</v>
@@ -6549,7 +6558,7 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B396" t="s">
         <v>99</v>
@@ -6563,10 +6572,10 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B397" t="s">
-        <v>171</v>
+        <v>12</v>
       </c>
       <c r="C397" t="b">
         <v>0</v>
@@ -6577,13 +6586,13 @@
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B398" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C398" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D398" t="s">
         <v>6</v>
@@ -6591,44 +6600,44 @@
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B399" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="C399" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D399" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B400" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C400" t="b">
         <v>0</v>
       </c>
       <c r="D400" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B401" t="s">
-        <v>34</v>
+        <v>98</v>
       </c>
       <c r="C401" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D401" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
@@ -6636,21 +6645,21 @@
         <v>170</v>
       </c>
       <c r="B402" t="s">
-        <v>31</v>
+        <v>97</v>
       </c>
       <c r="C402" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D402" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B403" t="s">
-        <v>160</v>
+        <v>115</v>
       </c>
       <c r="C403" t="b">
         <v>0</v>
@@ -6661,69 +6670,69 @@
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B404" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="C404" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D404" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B405" t="s">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="C405" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D405" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B406" t="s">
-        <v>34</v>
+        <v>115</v>
       </c>
       <c r="C406" t="b">
         <v>0</v>
       </c>
       <c r="D406" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B407" t="s">
-        <v>31</v>
+        <v>99</v>
       </c>
       <c r="C407" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D407" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B408" t="s">
-        <v>13</v>
+        <v>97</v>
       </c>
       <c r="C408" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D408" t="s">
         <v>6</v>
@@ -6731,10 +6740,10 @@
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B409" t="s">
-        <v>10</v>
+        <v>115</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
@@ -6745,16 +6754,16 @@
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B410" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="C410" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D410" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
@@ -6762,13 +6771,13 @@
         <v>173</v>
       </c>
       <c r="B411" t="s">
-        <v>32</v>
+        <v>174</v>
       </c>
       <c r="C411" t="b">
         <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
@@ -6776,13 +6785,13 @@
         <v>173</v>
       </c>
       <c r="B412" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="C412" t="b">
         <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
@@ -6790,7 +6799,7 @@
         <v>173</v>
       </c>
       <c r="B413" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
@@ -6801,55 +6810,55 @@
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B414" t="s">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="C414" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D414" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B415" t="s">
-        <v>115</v>
+        <v>34</v>
       </c>
       <c r="C415" t="b">
         <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B416" t="s">
-        <v>175</v>
+        <v>31</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
       </c>
       <c r="D416" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B417" t="s">
-        <v>97</v>
+        <v>161</v>
       </c>
       <c r="C417" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D417" t="s">
         <v>6</v>
@@ -6857,69 +6866,69 @@
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B418" t="s">
-        <v>115</v>
+        <v>8</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
       </c>
       <c r="D418" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B419" t="s">
-        <v>175</v>
+        <v>32</v>
       </c>
       <c r="C419" t="b">
         <v>0</v>
       </c>
       <c r="D419" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B420" t="s">
-        <v>177</v>
+        <v>34</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
       </c>
       <c r="D420" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B421" t="s">
-        <v>179</v>
+        <v>31</v>
       </c>
       <c r="C421" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D421" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B422" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C422" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D422" t="s">
         <v>6</v>
@@ -6927,10 +6936,10 @@
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B423" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
@@ -6941,66 +6950,66 @@
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B424" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
       </c>
       <c r="D424" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B425" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C425" t="b">
         <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B426" t="s">
-        <v>180</v>
+        <v>34</v>
       </c>
       <c r="C426" t="b">
         <v>0</v>
       </c>
       <c r="D426" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B427" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C427" t="b">
         <v>0</v>
       </c>
       <c r="D427" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B428" t="s">
-        <v>182</v>
+        <v>97</v>
       </c>
       <c r="C428" t="b">
         <v>1</v>
@@ -7011,13 +7020,13 @@
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B429" t="s">
-        <v>179</v>
+        <v>115</v>
       </c>
       <c r="C429" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D429" t="s">
         <v>6</v>
@@ -7025,13 +7034,13 @@
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B430" t="s">
-        <v>10</v>
+        <v>178</v>
       </c>
       <c r="C430" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D430" t="s">
         <v>6</v>
@@ -7039,13 +7048,13 @@
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B431" t="s">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="C431" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D431" t="s">
         <v>6</v>
@@ -7053,44 +7062,44 @@
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B432" t="s">
-        <v>32</v>
+        <v>115</v>
       </c>
       <c r="C432" t="b">
         <v>0</v>
       </c>
       <c r="D432" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B433" t="s">
-        <v>8</v>
+        <v>178</v>
       </c>
       <c r="C433" t="b">
         <v>0</v>
       </c>
       <c r="D433" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B434" t="s">
-        <v>46</v>
+        <v>180</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
       </c>
       <c r="D434" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
@@ -7098,10 +7107,10 @@
         <v>181</v>
       </c>
       <c r="B435" t="s">
-        <v>38</v>
+        <v>182</v>
       </c>
       <c r="C435" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D435" t="s">
         <v>6</v>
@@ -7109,10 +7118,10 @@
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B436" t="s">
-        <v>183</v>
+        <v>10</v>
       </c>
       <c r="C436" t="b">
         <v>1</v>
@@ -7123,7 +7132,7 @@
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B437" t="s">
         <v>12</v>
@@ -7137,55 +7146,55 @@
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B438" t="s">
-        <v>185</v>
+        <v>32</v>
       </c>
       <c r="C438" t="b">
         <v>0</v>
       </c>
       <c r="D438" t="s">
-        <v>186</v>
+        <v>33</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B439" t="s">
-        <v>187</v>
+        <v>8</v>
       </c>
       <c r="C439" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D439" t="s">
-        <v>188</v>
+        <v>9</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B440" t="s">
-        <v>5</v>
+        <v>183</v>
       </c>
       <c r="C440" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D440" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B441" t="s">
-        <v>190</v>
+        <v>38</v>
       </c>
       <c r="C441" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D441" t="s">
         <v>6</v>
@@ -7193,10 +7202,10 @@
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="B442" t="s">
-        <v>5</v>
+        <v>185</v>
       </c>
       <c r="C442" t="b">
         <v>1</v>
@@ -7207,10 +7216,10 @@
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="B443" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="C443" t="b">
         <v>1</v>
@@ -7221,10 +7230,10 @@
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="B444" t="s">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="C444" t="b">
         <v>1</v>
@@ -7235,13 +7244,13 @@
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="B445" t="s">
-        <v>193</v>
+        <v>12</v>
       </c>
       <c r="C445" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D445" t="s">
         <v>6</v>
@@ -7249,55 +7258,55 @@
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="B446" t="s">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="C446" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D446" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="B447" t="s">
-        <v>195</v>
+        <v>8</v>
       </c>
       <c r="C447" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D447" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="B448" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C448" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D448" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="B449" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="C449" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D449" t="s">
         <v>6</v>
@@ -7305,10 +7314,10 @@
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>198</v>
+        <v>84</v>
       </c>
       <c r="B450" t="s">
-        <v>199</v>
+        <v>186</v>
       </c>
       <c r="C450" t="b">
         <v>1</v>
@@ -7319,13 +7328,13 @@
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>200</v>
+        <v>84</v>
       </c>
       <c r="B451" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C451" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D451" t="s">
         <v>6</v>
@@ -7333,41 +7342,41 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
       <c r="B452" t="s">
-        <v>201</v>
+        <v>188</v>
       </c>
       <c r="C452" t="b">
         <v>0</v>
       </c>
       <c r="D452" t="s">
-        <v>6</v>
+        <v>189</v>
       </c>
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="B453" t="s">
-        <v>5</v>
+        <v>190</v>
       </c>
       <c r="C453" t="b">
         <v>1</v>
       </c>
       <c r="D453" t="s">
-        <v>6</v>
+        <v>191</v>
       </c>
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="B454" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C454" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D454" t="s">
         <v>6</v>
@@ -7375,10 +7384,10 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="B455" t="s">
-        <v>5</v>
+        <v>193</v>
       </c>
       <c r="C455" t="b">
         <v>1</v>
@@ -7389,13 +7398,13 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="B456" t="s">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="C456" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D456" t="s">
         <v>6</v>
@@ -7403,10 +7412,10 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B457" t="s">
-        <v>5</v>
+        <v>193</v>
       </c>
       <c r="C457" t="b">
         <v>1</v>
@@ -7417,13 +7426,13 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="B458" t="s">
-        <v>201</v>
+        <v>97</v>
       </c>
       <c r="C458" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D458" t="s">
         <v>6</v>
@@ -7431,10 +7440,10 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="B459" t="s">
-        <v>5</v>
+        <v>196</v>
       </c>
       <c r="C459" t="b">
         <v>1</v>
@@ -7445,13 +7454,13 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="B460" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C460" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D460" t="s">
         <v>6</v>
@@ -7459,13 +7468,13 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="B461" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="C461" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D461" t="s">
         <v>6</v>
@@ -7473,13 +7482,13 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B462" t="s">
-        <v>179</v>
+        <v>5</v>
       </c>
       <c r="C462" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D462" t="s">
         <v>6</v>
@@ -7487,10 +7496,10 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B463" t="s">
-        <v>207</v>
+        <v>5</v>
       </c>
       <c r="C463" t="b">
         <v>1</v>
@@ -7501,13 +7510,13 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B464" t="s">
-        <v>12</v>
+        <v>202</v>
       </c>
       <c r="C464" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D464" t="s">
         <v>6</v>
@@ -7515,7 +7524,7 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B465" t="s">
         <v>5</v>
@@ -7529,10 +7538,10 @@
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B466" t="s">
-        <v>7</v>
+        <v>204</v>
       </c>
       <c r="C466" t="b">
         <v>0</v>
@@ -7543,27 +7552,27 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B467" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C467" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D467" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B468" t="s">
-        <v>10</v>
+        <v>204</v>
       </c>
       <c r="C468" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D468" t="s">
         <v>6</v>
@@ -7571,13 +7580,13 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B469" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C469" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7585,13 +7594,13 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B470" t="s">
-        <v>12</v>
+        <v>204</v>
       </c>
       <c r="C470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7599,10 +7608,10 @@
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B471" t="s">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="C471" t="b">
         <v>1</v>
@@ -7613,16 +7622,16 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B472" t="s">
-        <v>46</v>
+        <v>204</v>
       </c>
       <c r="C472" t="b">
         <v>0</v>
       </c>
       <c r="D472" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
@@ -7630,7 +7639,7 @@
         <v>208</v>
       </c>
       <c r="B473" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C473" t="b">
         <v>1</v>
@@ -7641,10 +7650,10 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B474" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C474" t="b">
         <v>0</v>
@@ -7655,13 +7664,13 @@
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B475" t="s">
-        <v>38</v>
+        <v>185</v>
       </c>
       <c r="C475" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D475" t="s">
         <v>6</v>
@@ -7669,13 +7678,13 @@
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B476" t="s">
-        <v>52</v>
+        <v>182</v>
       </c>
       <c r="C476" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D476" t="s">
         <v>6</v>
@@ -7683,57 +7692,253 @@
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B477" t="s">
-        <v>19</v>
+        <v>210</v>
       </c>
       <c r="C477" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D477" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B478" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="C478" t="b">
         <v>0</v>
       </c>
       <c r="D478" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B479" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C479" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D479" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B480" t="s">
+        <v>7</v>
+      </c>
+      <c r="C480" t="b">
+        <v>0</v>
+      </c>
+      <c r="D480" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="481" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A481" t="s">
+        <v>211</v>
+      </c>
+      <c r="B481" t="s">
+        <v>8</v>
+      </c>
+      <c r="C481" t="b">
+        <v>0</v>
+      </c>
+      <c r="D481" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A482" t="s">
+        <v>211</v>
+      </c>
+      <c r="B482" t="s">
+        <v>10</v>
+      </c>
+      <c r="C482" t="b">
+        <v>1</v>
+      </c>
+      <c r="D482" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="483" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A483" t="s">
+        <v>211</v>
+      </c>
+      <c r="B483" t="s">
+        <v>11</v>
+      </c>
+      <c r="C483" t="b">
+        <v>0</v>
+      </c>
+      <c r="D483" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="484" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A484" t="s">
+        <v>211</v>
+      </c>
+      <c r="B484" t="s">
+        <v>12</v>
+      </c>
+      <c r="C484" t="b">
+        <v>1</v>
+      </c>
+      <c r="D484" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="485" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A485" t="s">
+        <v>211</v>
+      </c>
+      <c r="B485" t="s">
+        <v>45</v>
+      </c>
+      <c r="C485" t="b">
+        <v>1</v>
+      </c>
+      <c r="D485" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="486" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A486" t="s">
+        <v>211</v>
+      </c>
+      <c r="B486" t="s">
+        <v>46</v>
+      </c>
+      <c r="C486" t="b">
+        <v>0</v>
+      </c>
+      <c r="D486" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="487" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A487" t="s">
+        <v>211</v>
+      </c>
+      <c r="B487" t="s">
+        <v>13</v>
+      </c>
+      <c r="C487" t="b">
+        <v>1</v>
+      </c>
+      <c r="D487" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A488" t="s">
+        <v>211</v>
+      </c>
+      <c r="B488" t="s">
+        <v>37</v>
+      </c>
+      <c r="C488" t="b">
+        <v>0</v>
+      </c>
+      <c r="D488" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A489" t="s">
+        <v>211</v>
+      </c>
+      <c r="B489" t="s">
+        <v>38</v>
+      </c>
+      <c r="C489" t="b">
+        <v>1</v>
+      </c>
+      <c r="D489" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="490" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A490" t="s">
+        <v>211</v>
+      </c>
+      <c r="B490" t="s">
+        <v>52</v>
+      </c>
+      <c r="C490" t="b">
+        <v>1</v>
+      </c>
+      <c r="D490" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="491" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A491" t="s">
+        <v>211</v>
+      </c>
+      <c r="B491" t="s">
+        <v>19</v>
+      </c>
+      <c r="C491" t="b">
+        <v>0</v>
+      </c>
+      <c r="D491" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="492" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A492" t="s">
+        <v>211</v>
+      </c>
+      <c r="B492" t="s">
+        <v>31</v>
+      </c>
+      <c r="C492" t="b">
+        <v>0</v>
+      </c>
+      <c r="D492" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="493" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A493" t="s">
+        <v>211</v>
+      </c>
+      <c r="B493" t="s">
+        <v>32</v>
+      </c>
+      <c r="C493" t="b">
+        <v>0</v>
+      </c>
+      <c r="D493" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="494" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A494" t="s">
+        <v>211</v>
+      </c>
+      <c r="B494" t="s">
         <v>34</v>
       </c>
-      <c r="C480" t="b">
-        <v>0</v>
-      </c>
-      <c r="D480" t="s">
+      <c r="C494" t="b">
+        <v>0</v>
+      </c>
+      <c r="D494" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>